<commit_message>
Revert "Update drainage sheet for J01 junction and RP03 rename"
This reverts commit c86ab2f93c9b99cc97627b689937bdf602e10e5b.
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple.xlsx
+++ b/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple.xlsx
@@ -185,7 +185,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -251,16 +251,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -765,7 +755,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="464">
+  <cellXfs count="448">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2052,54 +2042,6 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="8" fillId="14" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="13" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="13" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="14" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="14" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="13" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="13" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="14" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="13" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="14" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="13" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="13" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2181,6 +2123,52 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="twoCell">
+    <from>
+      <col>0</col>
+      <colOff>222120</colOff>
+      <row>1</row>
+      <rowOff>63360</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>459360</colOff>
+      <row>4</row>
+      <rowOff>42480</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="0" name="Picture 1" descr="Marchand_Houle_RGB"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="222120" y="415800"/>
+          <a:ext cx="2980440" cy="874440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525">
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2364,7 +2352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.50390625" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="110" customWidth="1" style="205" min="1" max="1"/>
@@ -2373,7 +2361,7 @@
     <row r="1" ht="17.35" customHeight="1" s="206">
       <c r="A1" s="207" t="inlineStr">
         <is>
-          <t>Adaptation méthode simple Saint-Hubert ← données projet + plan J01/RP03 (Olivier)</t>
+          <t>Adaptation méthode simple Saint-Hubert ← données Reseau_pluvial_dimensionnement_v1</t>
         </is>
       </c>
     </row>
@@ -2521,90 +2509,6 @@
       <c r="A27" s="205" t="inlineStr">
         <is>
           <t>4) Comparer rapidement aux diamètres du classeur v1 si désiré</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="205" t="inlineStr">
-        <is>
-          <t>MAJ 2026-07-31 (plan / Olivier):</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="205" t="inlineStr">
-        <is>
-          <t>- Nouveau regard J01; conduite L12 P02→J01 ≈ 1.4 m</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="205" t="inlineStr">
-        <is>
-          <t>- P03 renommé RP03; L01=P01→J01; L02=J01→RP03; L03=RP03→P10</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="205" t="inlineStr">
-        <is>
-          <t>- Longueurs corrigées selon étiquettes plan; H/I corrigés aux confluences P06 et J01</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="205" t="inlineStr">
-        <is>
-          <t>- Tronçon P12→RACC (9.6 m) ajouté</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="205" t="inlineStr">
-        <is>
-          <t>Fichier source utilisateur mentionné: Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx (non reçu dans l’environnement cloud — mis à jour depuis le plan).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>MAJ 2026-07-31 (plan / Olivier):</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>- Nouveau regard J01; conduite L12 P02→J01 ≈ 1.4 m</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>- P03 renommé RP03; L01=P01→J01; L02=J01→RP03; L03=RP03→P10</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>- Longueurs/diamètres corrigés selon étiquettes plan; H/I corrigés aux confluences P06 et J01</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>- Tronçon P12→RACC (9.6 m) ajouté</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Note: fichier "OLIVIER TECH. MODIF.xlsx" non reçu dans le cloud — mise à jour faite depuis le plan + classeur ADAPTE existant.</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC177"/>
+  <dimension ref="A1:AC173"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.00390625" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="209" min="1" max="1"/>
@@ -2683,7 +2587,7 @@
       <c r="G2" s="218" t="n"/>
       <c r="H2" s="219" t="inlineStr">
         <is>
-          <t>Réseau pluvial – projet (J01 + RP03; longueurs plan / Olivier)</t>
+          <t>Réseau pluvial – projet (données Reseau_pluvial_dimensionnement_v1)</t>
         </is>
       </c>
       <c r="I2" s="219" t="n"/>
@@ -2766,7 +2670,7 @@
       <c r="L4" s="235" t="n"/>
       <c r="M4" s="243" t="inlineStr">
         <is>
-          <t>Réseau local → J01/RP03 → P12 / RACC / PUB</t>
+          <t>Réseau local → exutoire P12 / PUB</t>
         </is>
       </c>
       <c r="P4" s="236" t="n"/>
@@ -3431,7 +3335,7 @@
     <row r="17" ht="22.5" customHeight="1" s="206">
       <c r="A17" s="335" t="inlineStr">
         <is>
-          <t>Tronçons (amont → aval) — topologie plan: P02→J01 (1.4 m); P03 renommé RP03</t>
+          <t>Tronçons (amont → aval) — données projet</t>
         </is>
       </c>
       <c r="B17" s="323" t="n"/>
@@ -3477,89 +3381,88 @@
           <t>P06</t>
         </is>
       </c>
-      <c r="D18" s="448">
+      <c r="D18" s="339">
         <f>'Temps de concentration'!B7</f>
         <v/>
       </c>
-      <c r="E18" s="449" t="n">
-        <v>0.044675</v>
-      </c>
-      <c r="F18" s="450" t="n">
+      <c r="E18" s="340" t="n">
+        <v>0.0447</v>
+      </c>
+      <c r="F18" s="341" t="n">
         <v>0.425</v>
       </c>
-      <c r="G18" s="451">
+      <c r="G18" s="342">
         <f>E18*F18</f>
         <v/>
       </c>
-      <c r="H18" s="451">
+      <c r="H18" s="342">
         <f>E18</f>
         <v/>
       </c>
-      <c r="I18" s="451">
+      <c r="I18" s="342">
         <f>G18</f>
         <v/>
       </c>
-      <c r="J18" s="452">
+      <c r="J18" s="343">
         <f>IF(H18=0,0,I18/H18)</f>
         <v/>
       </c>
-      <c r="K18" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D18+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D18+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D18+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D18+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D18+$S$9)^$T$9),$R$10/((D18+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L18" s="452">
+      <c r="K18" s="339">
+        <f>IF($S$2=0.5,$R$5/((D18+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D18+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D18+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D18+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D18+$S$9)^$T$9),$R$10/((D18+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L18" s="343">
         <f>0.00275*H18*J18*K18</f>
         <v/>
       </c>
-      <c r="M18" s="449" t="n">
-        <v>0.0308</v>
-      </c>
-      <c r="N18" s="453" t="n">
+      <c r="M18" s="340" t="n">
+        <v>0.0306</v>
+      </c>
+      <c r="N18" s="344" t="n">
         <v>200</v>
       </c>
-      <c r="O18" s="448">
+      <c r="O18" s="339">
         <f>IF(OR(N18&lt;=0,M18&lt;=0),0,((N18/4000)^(2/3)*SQRT(M18))/$S$11)</f>
         <v/>
       </c>
-      <c r="P18" s="454" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="Q18" s="448">
+      <c r="P18" s="345" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="Q18" s="339">
         <f>IF(O18=0,0,P18/(O18*60))</f>
         <v/>
       </c>
-      <c r="R18" s="452">
+      <c r="R18" s="343">
         <f>O18*(PI()*(N18/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S18" s="455" t="n">
+      <c r="S18" s="346" t="n">
         <v>17.62</v>
       </c>
-      <c r="T18" s="455" t="n">
+      <c r="T18" s="346" t="n">
         <v>17.14</v>
       </c>
-      <c r="U18" s="455" t="n">
-        <v>16.601</v>
-      </c>
-      <c r="V18" s="455" t="n">
-        <v>16.445</v>
-      </c>
-      <c r="W18" s="452">
+      <c r="U18" s="346" t="n">
+        <v>16.918</v>
+      </c>
+      <c r="V18" s="346" t="n">
+        <v>16.438</v>
+      </c>
+      <c r="W18" s="343">
         <f>S18-U18-N18/1000</f>
         <v/>
       </c>
-      <c r="X18" s="452">
+      <c r="X18" s="343">
         <f>T18-V18-N18/1000</f>
         <v/>
       </c>
-      <c r="Y18" s="452">
+      <c r="Y18" s="343">
         <f>P18*PI()*(N18/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z18" s="326" t="n"/>
       <c r="AA18" s="347" t="n"/>
-      <c r="AB18" s="456">
+      <c r="AB18" s="348">
         <f>IF(R18&gt;L18,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3585,89 +3488,88 @@
           <t>P06</t>
         </is>
       </c>
-      <c r="D19" s="448">
+      <c r="D19" s="339">
         <f>MAX('Temps de concentration'!C7, D18+Q18)</f>
         <v/>
       </c>
-      <c r="E19" s="449" t="n">
-        <v>0.044235</v>
-      </c>
-      <c r="F19" s="450" t="n">
+      <c r="E19" s="340" t="n">
+        <v>0.0442</v>
+      </c>
+      <c r="F19" s="341" t="n">
         <v>0.765</v>
       </c>
-      <c r="G19" s="451">
+      <c r="G19" s="342">
         <f>E19*F19</f>
         <v/>
       </c>
-      <c r="H19" s="451">
-        <f>E19</f>
-        <v/>
-      </c>
-      <c r="I19" s="451">
-        <f>G19</f>
-        <v/>
-      </c>
-      <c r="J19" s="452">
+      <c r="H19" s="342">
+        <f>H18+E19</f>
+        <v/>
+      </c>
+      <c r="I19" s="342">
+        <f>I18+G19</f>
+        <v/>
+      </c>
+      <c r="J19" s="343">
         <f>IF(H19=0,0,I19/H19)</f>
         <v/>
       </c>
-      <c r="K19" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D19+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D19+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D19+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D19+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D19+$S$9)^$T$9),$R$10/((D19+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L19" s="452">
+      <c r="K19" s="339">
+        <f>IF($S$2=0.5,$R$5/((D19+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D19+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D19+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D19+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D19+$S$9)^$T$9),$R$10/((D19+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L19" s="343">
         <f>0.00275*H19*J19*K19</f>
         <v/>
       </c>
-      <c r="M19" s="449" t="n">
+      <c r="M19" s="340" t="n">
         <v>0.01</v>
       </c>
-      <c r="N19" s="453" t="n">
-        <v>250</v>
-      </c>
-      <c r="O19" s="448">
+      <c r="N19" s="344" t="n">
+        <v>200</v>
+      </c>
+      <c r="O19" s="339">
         <f>IF(OR(N19&lt;=0,M19&lt;=0),0,((N19/4000)^(2/3)*SQRT(M19))/$S$11)</f>
         <v/>
       </c>
-      <c r="P19" s="454" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="Q19" s="448">
+      <c r="P19" s="345" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="Q19" s="339">
         <f>IF(O19=0,0,P19/(O19*60))</f>
         <v/>
       </c>
-      <c r="R19" s="452">
+      <c r="R19" s="343">
         <f>O19*(PI()*(N19/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S19" s="455" t="n">
+      <c r="S19" s="346" t="n">
         <v>17.09</v>
       </c>
-      <c r="T19" s="455" t="n">
+      <c r="T19" s="346" t="n">
         <v>17.14</v>
       </c>
-      <c r="U19" s="455" t="n">
-        <v>16.554</v>
-      </c>
-      <c r="V19" s="455" t="n">
-        <v>16.445</v>
-      </c>
-      <c r="W19" s="452">
+      <c r="U19" s="346" t="n">
+        <v>16.418</v>
+      </c>
+      <c r="V19" s="346" t="n">
+        <v>16.296</v>
+      </c>
+      <c r="W19" s="343">
         <f>S19-U19-N19/1000</f>
         <v/>
       </c>
-      <c r="X19" s="452">
+      <c r="X19" s="343">
         <f>T19-V19-N19/1000</f>
         <v/>
       </c>
-      <c r="Y19" s="452">
+      <c r="Y19" s="343">
         <f>P19*PI()*(N19/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z19" s="326" t="n"/>
       <c r="AA19" s="347" t="n"/>
-      <c r="AB19" s="456">
+      <c r="AB19" s="348">
         <f>IF(R19&gt;L19,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3693,89 +3595,88 @@
           <t>P04</t>
         </is>
       </c>
-      <c r="D20" s="448">
-        <f>MAX('Temps de concentration'!D7, MAX(D18+Q18,D19+Q19))</f>
-        <v/>
-      </c>
-      <c r="E20" s="449" t="n">
-        <v>0.01479</v>
-      </c>
-      <c r="F20" s="450" t="n">
+      <c r="D20" s="339">
+        <f>MAX('Temps de concentration'!D7, D19+Q19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="340" t="n">
+        <v>0.0148</v>
+      </c>
+      <c r="F20" s="341" t="n">
         <v>0.6840000000000001</v>
       </c>
-      <c r="G20" s="451">
+      <c r="G20" s="342">
         <f>E20*F20</f>
         <v/>
       </c>
-      <c r="H20" s="451">
-        <f>H18+H19+E20</f>
-        <v/>
-      </c>
-      <c r="I20" s="451">
-        <f>I18+I19+G20</f>
-        <v/>
-      </c>
-      <c r="J20" s="452">
+      <c r="H20" s="342">
+        <f>H19+E20</f>
+        <v/>
+      </c>
+      <c r="I20" s="342">
+        <f>I19+G20</f>
+        <v/>
+      </c>
+      <c r="J20" s="343">
         <f>IF(H20=0,0,I20/H20)</f>
         <v/>
       </c>
-      <c r="K20" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D20+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D20+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D20+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D20+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D20+$S$9)^$T$9),$R$10/((D20+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L20" s="452">
+      <c r="K20" s="339">
+        <f>IF($S$2=0.5,$R$5/((D20+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D20+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D20+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D20+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D20+$S$9)^$T$9),$R$10/((D20+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L20" s="343">
         <f>0.00275*H20*J20*K20</f>
         <v/>
       </c>
-      <c r="M20" s="449" t="n">
+      <c r="M20" s="340" t="n">
         <v>0.01</v>
       </c>
-      <c r="N20" s="453" t="n">
-        <v>250</v>
-      </c>
-      <c r="O20" s="448">
+      <c r="N20" s="344" t="n">
+        <v>200</v>
+      </c>
+      <c r="O20" s="339">
         <f>IF(OR(N20&lt;=0,M20&lt;=0),0,((N20/4000)^(2/3)*SQRT(M20))/$S$11)</f>
         <v/>
       </c>
-      <c r="P20" s="454" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="Q20" s="448">
+      <c r="P20" s="345" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="Q20" s="339">
         <f>IF(O20=0,0,P20/(O20*60))</f>
         <v/>
       </c>
-      <c r="R20" s="452">
+      <c r="R20" s="343">
         <f>O20*(PI()*(N20/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S20" s="455" t="n">
+      <c r="S20" s="346" t="n">
         <v>17.14</v>
       </c>
-      <c r="T20" s="455" t="n">
+      <c r="T20" s="346" t="n">
         <v>17.28</v>
       </c>
-      <c r="U20" s="455" t="n">
-        <v>16.425</v>
-      </c>
-      <c r="V20" s="455" t="n">
-        <v>16.273</v>
-      </c>
-      <c r="W20" s="452">
+      <c r="U20" s="346" t="n">
+        <v>16.276</v>
+      </c>
+      <c r="V20" s="346" t="n">
+        <v>16.18</v>
+      </c>
+      <c r="W20" s="343">
         <f>S20-U20-N20/1000</f>
         <v/>
       </c>
-      <c r="X20" s="452">
+      <c r="X20" s="343">
         <f>T20-V20-N20/1000</f>
         <v/>
       </c>
-      <c r="Y20" s="452">
+      <c r="Y20" s="343">
         <f>P20*PI()*(N20/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z20" s="326" t="n"/>
       <c r="AA20" s="347" t="n"/>
-      <c r="AB20" s="456">
+      <c r="AB20" s="348">
         <f>IF(R20&gt;L20,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3801,89 +3702,88 @@
           <t>P01</t>
         </is>
       </c>
-      <c r="D21" s="448">
+      <c r="D21" s="339">
         <f>MAX('Temps de concentration'!E7, D20+Q20)</f>
         <v/>
       </c>
-      <c r="E21" s="449" t="n">
-        <v>0.00945</v>
-      </c>
-      <c r="F21" s="450" t="n">
+      <c r="E21" s="340" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="F21" s="341" t="n">
         <v>0.547</v>
       </c>
-      <c r="G21" s="451">
+      <c r="G21" s="342">
         <f>E21*F21</f>
         <v/>
       </c>
-      <c r="H21" s="451">
+      <c r="H21" s="342">
         <f>H20+E21</f>
         <v/>
       </c>
-      <c r="I21" s="451">
+      <c r="I21" s="342">
         <f>I20+G21</f>
         <v/>
       </c>
-      <c r="J21" s="452">
+      <c r="J21" s="343">
         <f>IF(H21=0,0,I21/H21)</f>
         <v/>
       </c>
-      <c r="K21" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D21+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D21+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D21+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D21+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D21+$S$9)^$T$9),$R$10/((D21+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L21" s="452">
+      <c r="K21" s="339">
+        <f>IF($S$2=0.5,$R$5/((D21+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D21+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D21+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D21+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D21+$S$9)^$T$9),$R$10/((D21+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L21" s="343">
         <f>0.00275*H21*J21*K21</f>
         <v/>
       </c>
-      <c r="M21" s="449" t="n">
+      <c r="M21" s="340" t="n">
         <v>0.01</v>
       </c>
-      <c r="N21" s="453" t="n">
+      <c r="N21" s="344" t="n">
         <v>250</v>
       </c>
-      <c r="O21" s="448">
+      <c r="O21" s="339">
         <f>IF(OR(N21&lt;=0,M21&lt;=0),0,((N21/4000)^(2/3)*SQRT(M21))/$S$11)</f>
         <v/>
       </c>
-      <c r="P21" s="454" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="Q21" s="448">
+      <c r="P21" s="345" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="Q21" s="339">
         <f>IF(O21=0,0,P21/(O21*60))</f>
         <v/>
       </c>
-      <c r="R21" s="452">
+      <c r="R21" s="343">
         <f>O21*(PI()*(N21/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S21" s="455" t="n">
+      <c r="S21" s="346" t="n">
         <v>17.28</v>
       </c>
-      <c r="T21" s="455" t="n">
-        <v>17.23</v>
-      </c>
-      <c r="U21" s="455" t="n">
-        <v>16.253</v>
-      </c>
-      <c r="V21" s="455" t="n">
-        <v>16.114</v>
-      </c>
-      <c r="W21" s="452">
+      <c r="T21" s="346" t="n">
+        <v>17.237</v>
+      </c>
+      <c r="U21" s="346" t="n">
+        <v>16.16</v>
+      </c>
+      <c r="V21" s="346" t="n">
+        <v>16.025</v>
+      </c>
+      <c r="W21" s="343">
         <f>S21-U21-N21/1000</f>
         <v/>
       </c>
-      <c r="X21" s="452">
+      <c r="X21" s="343">
         <f>T21-V21-N21/1000</f>
         <v/>
       </c>
-      <c r="Y21" s="452">
+      <c r="Y21" s="343">
         <f>P21*PI()*(N21/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z21" s="326" t="n"/>
       <c r="AA21" s="347" t="n"/>
-      <c r="AB21" s="456">
+      <c r="AB21" s="348">
         <f>IF(R21&gt;L21,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3906,98 +3806,97 @@
       </c>
       <c r="C22" s="338" t="inlineStr">
         <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="D22" s="448">
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="D22" s="339">
         <f>MAX('Temps de concentration'!F7, D21+Q21)</f>
         <v/>
       </c>
-      <c r="E22" s="449" t="n">
-        <v>0.02573</v>
-      </c>
-      <c r="F22" s="450" t="n">
+      <c r="E22" s="340" t="n">
+        <v>0.0257</v>
+      </c>
+      <c r="F22" s="341" t="n">
         <v>0.633</v>
       </c>
-      <c r="G22" s="451">
+      <c r="G22" s="342">
         <f>E22*F22</f>
         <v/>
       </c>
-      <c r="H22" s="451">
+      <c r="H22" s="342">
         <f>H21+E22</f>
         <v/>
       </c>
-      <c r="I22" s="451">
+      <c r="I22" s="342">
         <f>I21+G22</f>
         <v/>
       </c>
-      <c r="J22" s="452">
+      <c r="J22" s="343">
         <f>IF(H22=0,0,I22/H22)</f>
         <v/>
       </c>
-      <c r="K22" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D22+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D22+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D22+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D22+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D22+$S$9)^$T$9),$R$10/((D22+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L22" s="452">
+      <c r="K22" s="339">
+        <f>IF($S$2=0.5,$R$5/((D22+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D22+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D22+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D22+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D22+$S$9)^$T$9),$R$10/((D22+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L22" s="343">
         <f>0.00275*H22*J22*K22</f>
         <v/>
       </c>
-      <c r="M22" s="449" t="n">
+      <c r="M22" s="340" t="n">
         <v>0.01</v>
       </c>
-      <c r="N22" s="453" t="n">
-        <v>300</v>
-      </c>
-      <c r="O22" s="448">
+      <c r="N22" s="344" t="n">
+        <v>250</v>
+      </c>
+      <c r="O22" s="339">
         <f>IF(OR(N22&lt;=0,M22&lt;=0),0,((N22/4000)^(2/3)*SQRT(M22))/$S$11)</f>
         <v/>
       </c>
-      <c r="P22" s="454" t="n">
+      <c r="P22" s="345" t="n">
         <v>14.2</v>
       </c>
-      <c r="Q22" s="448">
+      <c r="Q22" s="339">
         <f>IF(O22=0,0,P22/(O22*60))</f>
         <v/>
       </c>
-      <c r="R22" s="452">
+      <c r="R22" s="343">
         <f>O22*(PI()*(N22/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S22" s="455" t="n">
-        <v>17.23</v>
-      </c>
-      <c r="T22" s="455" t="n">
-        <v>17.12</v>
-      </c>
-      <c r="U22" s="455" t="n">
-        <v>16.094</v>
-      </c>
-      <c r="V22" s="455" t="n">
-        <v>15.952</v>
-      </c>
-      <c r="W22" s="452">
+      <c r="S22" s="346" t="n">
+        <v>17.237</v>
+      </c>
+      <c r="T22" s="346" t="n">
+        <v>17.131</v>
+      </c>
+      <c r="U22" s="346" t="n">
+        <v>16.005</v>
+      </c>
+      <c r="V22" s="346" t="n">
+        <v>15.863</v>
+      </c>
+      <c r="W22" s="343">
         <f>S22-U22-N22/1000</f>
         <v/>
       </c>
-      <c r="X22" s="452">
+      <c r="X22" s="343">
         <f>T22-V22-N22/1000</f>
         <v/>
       </c>
-      <c r="Y22" s="452">
+      <c r="Y22" s="343">
         <f>P22*PI()*(N22/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z22" s="326" t="n"/>
       <c r="AA22" s="347" t="n"/>
-      <c r="AB22" s="456">
+      <c r="AB22" s="348">
         <f>IF(R22&gt;L22,"OK","AUGMENTER D")</f>
         <v/>
       </c>
       <c r="AC22" s="349" t="inlineStr">
         <is>
-          <t>L01_P01_J01</t>
+          <t>L01_P01_P02</t>
         </is>
       </c>
     </row>
@@ -4014,105 +3913,104 @@
       </c>
       <c r="C23" s="338" t="inlineStr">
         <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="D23" s="448">
-        <f>'Temps de concentration'!J7</f>
-        <v/>
-      </c>
-      <c r="E23" s="449" t="n">
-        <v>0.01228</v>
-      </c>
-      <c r="F23" s="450" t="n">
-        <v>0.672</v>
-      </c>
-      <c r="G23" s="451">
+          <t>P03</t>
+        </is>
+      </c>
+      <c r="D23" s="339">
+        <f>MAX('Temps de concentration'!G7, D22+Q22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="340" t="n">
+        <v>0.0468</v>
+      </c>
+      <c r="F23" s="341" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="G23" s="342">
         <f>E23*F23</f>
         <v/>
       </c>
-      <c r="H23" s="451">
-        <f>E23</f>
-        <v/>
-      </c>
-      <c r="I23" s="451">
-        <f>G23</f>
-        <v/>
-      </c>
-      <c r="J23" s="452">
+      <c r="H23" s="342">
+        <f>H22+E23</f>
+        <v/>
+      </c>
+      <c r="I23" s="342">
+        <f>I22+G23</f>
+        <v/>
+      </c>
+      <c r="J23" s="343">
         <f>IF(H23=0,0,I23/H23)</f>
         <v/>
       </c>
-      <c r="K23" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D23+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D23+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D23+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D23+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D23+$S$9)^$T$9),$R$10/((D23+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L23" s="452">
+      <c r="K23" s="339">
+        <f>IF($S$2=0.5,$R$5/((D23+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D23+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D23+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D23+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D23+$S$9)^$T$9),$R$10/((D23+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L23" s="343">
         <f>0.00275*H23*J23*K23</f>
         <v/>
       </c>
-      <c r="M23" s="449" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="N23" s="453" t="n">
-        <v>300</v>
-      </c>
-      <c r="O23" s="448">
+      <c r="M23" s="340" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="N23" s="344" t="n">
+        <v>250</v>
+      </c>
+      <c r="O23" s="339">
         <f>IF(OR(N23&lt;=0,M23&lt;=0),0,((N23/4000)^(2/3)*SQRT(M23))/$S$11)</f>
         <v/>
       </c>
-      <c r="P23" s="454" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="Q23" s="448">
+      <c r="P23" s="345" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="Q23" s="339">
         <f>IF(O23=0,0,P23/(O23*60))</f>
         <v/>
       </c>
-      <c r="R23" s="452">
+      <c r="R23" s="343">
         <f>O23*(PI()*(N23/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S23" s="455" t="n">
+      <c r="S23" s="346" t="n">
         <v>17.131</v>
       </c>
-      <c r="T23" s="455" t="n">
-        <v>17.12</v>
-      </c>
-      <c r="U23" s="455" t="n">
-        <v>15.946</v>
-      </c>
-      <c r="V23" s="455" t="n">
-        <v>15.932</v>
-      </c>
-      <c r="W23" s="452">
+      <c r="T23" s="346" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="U23" s="346" t="n">
+        <v>15.843</v>
+      </c>
+      <c r="V23" s="346" t="n">
+        <v>15.722</v>
+      </c>
+      <c r="W23" s="343">
         <f>S23-U23-N23/1000</f>
         <v/>
       </c>
-      <c r="X23" s="452">
+      <c r="X23" s="343">
         <f>T23-V23-N23/1000</f>
         <v/>
       </c>
-      <c r="Y23" s="452">
+      <c r="Y23" s="343">
         <f>P23*PI()*(N23/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z23" s="326" t="n"/>
       <c r="AA23" s="347" t="n"/>
-      <c r="AB23" s="456">
+      <c r="AB23" s="348">
         <f>IF(R23&gt;L23,"OK","AUGMENTER D")</f>
         <v/>
       </c>
       <c r="AC23" s="349" t="inlineStr">
         <is>
-          <t>L12_P02_J01</t>
+          <t>L02_P02_P03</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22.5" customHeight="1" s="206">
       <c r="A24" s="338" t="inlineStr">
         <is>
-          <t>J01</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="B24" s="338" t="inlineStr">
@@ -4122,105 +4020,104 @@
       </c>
       <c r="C24" s="338" t="inlineStr">
         <is>
-          <t>RP03</t>
-        </is>
-      </c>
-      <c r="D24" s="448">
-        <f>MAX('Temps de concentration'!G7, MAX(D22+Q22,D23+Q23))</f>
-        <v/>
-      </c>
-      <c r="E24" s="449" t="n">
-        <v>0.034509</v>
-      </c>
-      <c r="F24" s="450" t="n">
-        <v>0.631</v>
-      </c>
-      <c r="G24" s="451">
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D24" s="339">
+        <f>D23+Q23</f>
+        <v/>
+      </c>
+      <c r="E24" s="340" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="341" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G24" s="342">
         <f>E24*F24</f>
         <v/>
       </c>
-      <c r="H24" s="451">
-        <f>H22+H23+E24</f>
-        <v/>
-      </c>
-      <c r="I24" s="451">
-        <f>I22+I23+G24</f>
-        <v/>
-      </c>
-      <c r="J24" s="452">
+      <c r="H24" s="342">
+        <f>H23+E24</f>
+        <v/>
+      </c>
+      <c r="I24" s="342">
+        <f>I23+G24</f>
+        <v/>
+      </c>
+      <c r="J24" s="343">
         <f>IF(H24=0,0,I24/H24)</f>
         <v/>
       </c>
-      <c r="K24" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D24+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D24+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D24+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D24+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D24+$S$9)^$T$9),$R$10/((D24+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L24" s="452">
+      <c r="K24" s="339">
+        <f>IF($S$2=0.5,$R$5/((D24+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D24+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D24+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D24+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D24+$S$9)^$T$9),$R$10/((D24+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L24" s="343">
         <f>0.00275*H24*J24*K24</f>
         <v/>
       </c>
-      <c r="M24" s="449" t="n">
-        <v>0.0104</v>
-      </c>
-      <c r="N24" s="453" t="n">
-        <v>300</v>
-      </c>
-      <c r="O24" s="448">
+      <c r="M24" s="340" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N24" s="344" t="n">
+        <v>250</v>
+      </c>
+      <c r="O24" s="339">
         <f>IF(OR(N24&lt;=0,M24&lt;=0),0,((N24/4000)^(2/3)*SQRT(M24))/$S$11)</f>
         <v/>
       </c>
-      <c r="P24" s="454" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="Q24" s="448">
+      <c r="P24" s="345" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="Q24" s="339">
         <f>IF(O24=0,0,P24/(O24*60))</f>
         <v/>
       </c>
-      <c r="R24" s="452">
+      <c r="R24" s="343">
         <f>O24*(PI()*(N24/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S24" s="455" t="n">
-        <v>17.12</v>
-      </c>
-      <c r="T24" s="455" t="n">
+      <c r="S24" s="346" t="n">
         <v>17.01</v>
       </c>
-      <c r="U24" s="455" t="n">
-        <v>15.932</v>
-      </c>
-      <c r="V24" s="455" t="n">
-        <v>15.826</v>
-      </c>
-      <c r="W24" s="452">
+      <c r="T24" s="346" t="n">
+        <v>16.965</v>
+      </c>
+      <c r="U24" s="346" t="n">
+        <v>15.702</v>
+      </c>
+      <c r="V24" s="346" t="n">
+        <v>15.634</v>
+      </c>
+      <c r="W24" s="343">
         <f>S24-U24-N24/1000</f>
         <v/>
       </c>
-      <c r="X24" s="452">
+      <c r="X24" s="343">
         <f>T24-V24-N24/1000</f>
         <v/>
       </c>
-      <c r="Y24" s="452">
+      <c r="Y24" s="343">
         <f>P24*PI()*(N24/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z24" s="326" t="n"/>
       <c r="AA24" s="347" t="n"/>
-      <c r="AB24" s="456">
+      <c r="AB24" s="348">
         <f>IF(R24&gt;L24,"OK","AUGMENTER D")</f>
         <v/>
       </c>
       <c r="AC24" s="349" t="inlineStr">
         <is>
-          <t>L02_J01_RP03</t>
+          <t>L03_P03_P10</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22.5" customHeight="1" s="206">
       <c r="A25" s="338" t="inlineStr">
         <is>
-          <t>RP03</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="B25" s="338" t="inlineStr">
@@ -4230,105 +4127,104 @@
       </c>
       <c r="C25" s="338" t="inlineStr">
         <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="D25" s="448">
-        <f>D24+Q24</f>
-        <v/>
-      </c>
-      <c r="E25" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="450" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G25" s="451">
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D25" s="339">
+        <f>MAX('Temps de concentration'!H7, D24+Q24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="340" t="n">
+        <v>0.09030000000000001</v>
+      </c>
+      <c r="F25" s="341" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G25" s="342">
         <f>E25*F25</f>
         <v/>
       </c>
-      <c r="H25" s="451">
+      <c r="H25" s="342">
         <f>H24+E25</f>
         <v/>
       </c>
-      <c r="I25" s="451">
+      <c r="I25" s="342">
         <f>I24+G25</f>
         <v/>
       </c>
-      <c r="J25" s="452">
+      <c r="J25" s="343">
         <f>IF(H25=0,0,I25/H25)</f>
         <v/>
       </c>
-      <c r="K25" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D25+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D25+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D25+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D25+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D25+$S$9)^$T$9),$R$10/((D25+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L25" s="452">
+      <c r="K25" s="339">
+        <f>IF($S$2=0.5,$R$5/((D25+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D25+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D25+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D25+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D25+$S$9)^$T$9),$R$10/((D25+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L25" s="343">
         <f>0.00275*H25*J25*K25</f>
         <v/>
       </c>
-      <c r="M25" s="449" t="n">
+      <c r="M25" s="340" t="n">
         <v>0.01</v>
       </c>
-      <c r="N25" s="453" t="n">
-        <v>375</v>
-      </c>
-      <c r="O25" s="448">
+      <c r="N25" s="344" t="n">
+        <v>300</v>
+      </c>
+      <c r="O25" s="339">
         <f>IF(OR(N25&lt;=0,M25&lt;=0),0,((N25/4000)^(2/3)*SQRT(M25))/$S$11)</f>
         <v/>
       </c>
-      <c r="P25" s="454" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="Q25" s="448">
+      <c r="P25" s="345" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Q25" s="339">
         <f>IF(O25=0,0,P25/(O25*60))</f>
         <v/>
       </c>
-      <c r="R25" s="452">
+      <c r="R25" s="343">
         <f>O25*(PI()*(N25/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S25" s="455" t="n">
-        <v>17.01</v>
-      </c>
-      <c r="T25" s="455" t="n">
+      <c r="S25" s="346" t="n">
         <v>16.965</v>
       </c>
-      <c r="U25" s="455" t="n">
-        <v>15.806</v>
-      </c>
-      <c r="V25" s="455" t="n">
-        <v>15.717</v>
-      </c>
-      <c r="W25" s="452">
+      <c r="T25" s="346" t="n">
+        <v>16.874</v>
+      </c>
+      <c r="U25" s="346" t="n">
+        <v>15.614</v>
+      </c>
+      <c r="V25" s="346" t="n">
+        <v>15.469</v>
+      </c>
+      <c r="W25" s="343">
         <f>S25-U25-N25/1000</f>
         <v/>
       </c>
-      <c r="X25" s="452">
+      <c r="X25" s="343">
         <f>T25-V25-N25/1000</f>
         <v/>
       </c>
-      <c r="Y25" s="452">
+      <c r="Y25" s="343">
         <f>P25*PI()*(N25/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z25" s="326" t="n"/>
       <c r="AA25" s="347" t="n"/>
-      <c r="AB25" s="456">
+      <c r="AB25" s="348">
         <f>IF(R25&gt;L25,"OK","AUGMENTER D")</f>
         <v/>
       </c>
       <c r="AC25" s="349" t="inlineStr">
         <is>
-          <t>L03_RP03_P10</t>
+          <t>L10_P10_P11</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22.5" customHeight="1" s="206">
       <c r="A26" s="338" t="inlineStr">
         <is>
-          <t>P10</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="B26" s="338" t="inlineStr">
@@ -4338,546 +4234,245 @@
       </c>
       <c r="C26" s="338" t="inlineStr">
         <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="D26" s="448">
-        <f>MAX('Temps de concentration'!H7, D25+Q25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="449" t="n">
-        <v>0.09030000000000001</v>
-      </c>
-      <c r="F26" s="450" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="G26" s="451">
+          <t>PUB</t>
+        </is>
+      </c>
+      <c r="D26" s="339">
+        <f>MAX('Temps de concentration'!I7, D25+Q25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="340" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="F26" s="341" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="G26" s="342">
         <f>E26*F26</f>
         <v/>
       </c>
-      <c r="H26" s="451">
+      <c r="H26" s="342">
         <f>H25+E26</f>
         <v/>
       </c>
-      <c r="I26" s="451">
+      <c r="I26" s="342">
         <f>I25+G26</f>
         <v/>
       </c>
-      <c r="J26" s="452">
+      <c r="J26" s="343">
         <f>IF(H26=0,0,I26/H26)</f>
         <v/>
       </c>
-      <c r="K26" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D26+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D26+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D26+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D26+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D26+$S$9)^$T$9),$R$10/((D26+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L26" s="452">
+      <c r="K26" s="339">
+        <f>IF($S$2=0.5,$R$5/((D26+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D26+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D26+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D26+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D26+$S$9)^$T$9),$R$10/((D26+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L26" s="343">
         <f>0.00275*H26*J26*K26</f>
         <v/>
       </c>
-      <c r="M26" s="449" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="N26" s="453" t="n">
-        <v>375</v>
-      </c>
-      <c r="O26" s="448">
+      <c r="M26" s="340" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="N26" s="344" t="n">
+        <v>300</v>
+      </c>
+      <c r="O26" s="339">
         <f>IF(OR(N26&lt;=0,M26&lt;=0),0,((N26/4000)^(2/3)*SQRT(M26))/$S$11)</f>
         <v/>
       </c>
-      <c r="P26" s="454" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="Q26" s="448">
+      <c r="P26" s="345" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="Q26" s="339">
         <f>IF(O26=0,0,P26/(O26*60))</f>
         <v/>
       </c>
-      <c r="R26" s="452">
+      <c r="R26" s="343">
         <f>O26*(PI()*(N26/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S26" s="455" t="n">
-        <v>16.965</v>
-      </c>
-      <c r="T26" s="455" t="n">
+      <c r="S26" s="346" t="n">
         <v>16.874</v>
       </c>
-      <c r="U26" s="455" t="n">
-        <v>15.697</v>
-      </c>
-      <c r="V26" s="455" t="n">
-        <v>15.552</v>
-      </c>
-      <c r="W26" s="452">
+      <c r="T26" s="346" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="U26" s="346" t="n">
+        <v>15.449</v>
+      </c>
+      <c r="V26" s="346" t="n">
+        <v>15.305</v>
+      </c>
+      <c r="W26" s="343">
         <f>S26-U26-N26/1000</f>
         <v/>
       </c>
-      <c r="X26" s="452">
+      <c r="X26" s="343">
         <f>T26-V26-N26/1000</f>
         <v/>
       </c>
-      <c r="Y26" s="452">
+      <c r="Y26" s="343">
         <f>P26*PI()*(N26/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z26" s="326" t="n"/>
       <c r="AA26" s="347" t="n"/>
-      <c r="AB26" s="456">
+      <c r="AB26" s="348">
         <f>IF(R26&gt;L26,"OK","AUGMENTER D")</f>
         <v/>
       </c>
       <c r="AC26" s="349" t="inlineStr">
         <is>
-          <t>L10_P10_P11</t>
+          <t>L11_P11_P12</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22.5" customHeight="1" s="206">
-      <c r="A27" s="338" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="B27" s="338" t="inlineStr">
-        <is>
-          <t>@</t>
-        </is>
-      </c>
-      <c r="C27" s="338" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="D27" s="448">
-        <f>MAX('Temps de concentration'!I7, D26+Q26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="449" t="n">
-        <v>0.049761</v>
-      </c>
-      <c r="F27" s="450" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="G27" s="451">
-        <f>E27*F27</f>
-        <v/>
-      </c>
-      <c r="H27" s="451">
-        <f>H26+E27</f>
-        <v/>
-      </c>
-      <c r="I27" s="451">
-        <f>I26+G27</f>
-        <v/>
-      </c>
-      <c r="J27" s="452">
-        <f>IF(H27=0,0,I27/H27)</f>
-        <v/>
-      </c>
-      <c r="K27" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D27+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D27+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D27+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D27+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D27+$S$9)^$T$9),$R$10/((D27+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L27" s="452">
-        <f>0.00275*H27*J27*K27</f>
-        <v/>
-      </c>
-      <c r="M27" s="449" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="N27" s="453" t="n">
-        <v>450</v>
-      </c>
-      <c r="O27" s="448">
-        <f>IF(OR(N27&lt;=0,M27&lt;=0),0,((N27/4000)^(2/3)*SQRT(M27))/$S$11)</f>
-        <v/>
-      </c>
-      <c r="P27" s="454" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="Q27" s="448">
-        <f>IF(O27=0,0,P27/(O27*60))</f>
-        <v/>
-      </c>
-      <c r="R27" s="452">
-        <f>O27*(PI()*(N27/1000)^2/4)</f>
-        <v/>
-      </c>
-      <c r="S27" s="455" t="n">
-        <v>16.874</v>
-      </c>
-      <c r="T27" s="455" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="U27" s="455" t="n">
-        <v>15.532</v>
-      </c>
-      <c r="V27" s="455" t="n">
-        <v>15.421</v>
-      </c>
-      <c r="W27" s="452">
-        <f>S27-U27-N27/1000</f>
-        <v/>
-      </c>
-      <c r="X27" s="452">
-        <f>T27-V27-N27/1000</f>
-        <v/>
-      </c>
-      <c r="Y27" s="452">
-        <f>P27*PI()*(N27/1000)^2/4</f>
-        <v/>
-      </c>
+      <c r="A27" s="350" t="n"/>
+      <c r="B27" s="351" t="n"/>
+      <c r="C27" s="352" t="n"/>
+      <c r="D27" s="353" t="n"/>
+      <c r="E27" s="354" t="n"/>
+      <c r="F27" s="331" t="n"/>
+      <c r="G27" s="354" t="n"/>
+      <c r="H27" s="354" t="n"/>
+      <c r="I27" s="354" t="n"/>
+      <c r="J27" s="331" t="n"/>
+      <c r="K27" s="331" t="n"/>
+      <c r="L27" s="355" t="n"/>
+      <c r="M27" s="356" t="n"/>
+      <c r="N27" s="325" t="n"/>
+      <c r="O27" s="357" t="n"/>
+      <c r="P27" s="353" t="n"/>
+      <c r="Q27" s="331" t="n"/>
+      <c r="R27" s="355" t="n"/>
+      <c r="S27" s="331" t="n"/>
+      <c r="T27" s="331" t="n"/>
+      <c r="U27" s="326" t="n"/>
+      <c r="V27" s="358" t="n"/>
+      <c r="W27" s="336" t="n"/>
+      <c r="X27" s="326" t="n"/>
+      <c r="Y27" s="326" t="n"/>
       <c r="Z27" s="326" t="n"/>
       <c r="AA27" s="347" t="n"/>
-      <c r="AB27" s="456">
-        <f>IF(R27&gt;L27,"OK","AUGMENTER D")</f>
-        <v/>
-      </c>
-      <c r="AC27" s="349" t="inlineStr">
-        <is>
-          <t>L11_P11_P12</t>
-        </is>
-      </c>
+      <c r="AB27" s="359" t="n"/>
     </row>
     <row r="28" ht="22.5" customHeight="1" s="206">
-      <c r="A28" s="338" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B28" s="338" t="inlineStr">
-        <is>
-          <t>@</t>
-        </is>
-      </c>
-      <c r="C28" s="338" t="inlineStr">
-        <is>
-          <t>RACC</t>
-        </is>
-      </c>
-      <c r="D28" s="448">
-        <f>D27+Q27</f>
-        <v/>
-      </c>
-      <c r="E28" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="450" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G28" s="451">
-        <f>E28*F28</f>
-        <v/>
-      </c>
-      <c r="H28" s="451">
-        <f>H27+E28</f>
-        <v/>
-      </c>
-      <c r="I28" s="451">
-        <f>I27+G28</f>
-        <v/>
-      </c>
-      <c r="J28" s="452">
-        <f>IF(H28=0,0,I28/H28)</f>
-        <v/>
-      </c>
-      <c r="K28" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D28+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D28+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D28+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D28+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D28+$S$9)^$T$9),$R$10/((D28+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L28" s="452">
-        <f>0.00275*H28*J28*K28</f>
-        <v/>
-      </c>
-      <c r="M28" s="449" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="N28" s="453" t="n">
-        <v>450</v>
-      </c>
-      <c r="O28" s="448">
-        <f>IF(OR(N28&lt;=0,M28&lt;=0),0,((N28/4000)^(2/3)*SQRT(M28))/$S$11)</f>
-        <v/>
-      </c>
-      <c r="P28" s="454" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="Q28" s="448">
-        <f>IF(O28=0,0,P28/(O28*60))</f>
-        <v/>
-      </c>
-      <c r="R28" s="452">
-        <f>O28*(PI()*(N28/1000)^2/4)</f>
-        <v/>
-      </c>
-      <c r="S28" s="455" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="T28" s="455" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="U28" s="455" t="n">
-        <v>15.401</v>
-      </c>
-      <c r="V28" s="455" t="n">
-        <v>15.305</v>
-      </c>
-      <c r="W28" s="452">
-        <f>S28-U28-N28/1000</f>
-        <v/>
-      </c>
-      <c r="X28" s="452">
-        <f>T28-V28-N28/1000</f>
-        <v/>
-      </c>
-      <c r="Y28" s="452">
-        <f>P28*PI()*(N28/1000)^2/4</f>
-        <v/>
-      </c>
+      <c r="A28" s="350" t="n"/>
+      <c r="B28" s="351" t="n"/>
+      <c r="C28" s="352" t="n"/>
+      <c r="D28" s="353" t="n"/>
+      <c r="E28" s="354" t="n"/>
+      <c r="F28" s="331" t="n"/>
+      <c r="G28" s="354" t="n"/>
+      <c r="H28" s="354" t="n"/>
+      <c r="I28" s="354" t="n"/>
+      <c r="J28" s="331" t="n"/>
+      <c r="K28" s="331" t="n"/>
+      <c r="L28" s="355" t="n"/>
+      <c r="M28" s="356" t="n"/>
+      <c r="N28" s="325" t="n"/>
+      <c r="O28" s="357" t="n"/>
+      <c r="P28" s="353" t="n"/>
+      <c r="Q28" s="331" t="n"/>
+      <c r="R28" s="355" t="n"/>
+      <c r="S28" s="331" t="n"/>
+      <c r="T28" s="331" t="n"/>
+      <c r="U28" s="326" t="n"/>
+      <c r="V28" s="358" t="n"/>
+      <c r="W28" s="336" t="n"/>
+      <c r="X28" s="326" t="n"/>
+      <c r="Y28" s="326" t="n"/>
       <c r="Z28" s="326" t="n"/>
       <c r="AA28" s="347" t="n"/>
-      <c r="AB28" s="456">
-        <f>IF(R28&gt;L28,"OK","AUGMENTER D")</f>
-        <v/>
-      </c>
-      <c r="AC28" s="349" t="inlineStr">
-        <is>
-          <t>L13_P12_RACC</t>
-        </is>
-      </c>
+      <c r="AB28" s="359" t="n"/>
     </row>
     <row r="29" ht="22.5" customHeight="1" s="206">
-      <c r="A29" s="338" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="B29" s="338" t="inlineStr">
-        <is>
-          <t>@</t>
-        </is>
-      </c>
-      <c r="C29" s="338" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="D29" s="448">
-        <f>MAX('Temps de concentration'!I7, D26+Q26)</f>
-        <v/>
-      </c>
-      <c r="E29" s="449" t="n">
-        <v>0.049761</v>
-      </c>
-      <c r="F29" s="450" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="G29" s="451">
-        <f>E27*F27</f>
-        <v/>
-      </c>
-      <c r="H29" s="451">
-        <f>H26+E27</f>
-        <v/>
-      </c>
-      <c r="I29" s="451">
-        <f>I26+G27</f>
-        <v/>
-      </c>
-      <c r="J29" s="452">
-        <f>IF(H27=0,0,I27/H27)</f>
-        <v/>
-      </c>
-      <c r="K29" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D27+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D27+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D27+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D27+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D27+$S$9)^$T$9),$R$10/((D27+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L29" s="452">
-        <f>0.00275*H27*J27*K27</f>
-        <v/>
-      </c>
-      <c r="M29" s="449" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="N29" s="453" t="n">
-        <v>450</v>
-      </c>
-      <c r="O29" s="448">
-        <f>IF(OR(N27&lt;=0,M27&lt;=0),0,((N27/4000)^(2/3)*SQRT(M27))/$S$11)</f>
-        <v/>
-      </c>
-      <c r="P29" s="454" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="Q29" s="448">
-        <f>IF(O27=0,0,P27/(O27*60))</f>
-        <v/>
-      </c>
-      <c r="R29" s="452">
-        <f>O27*(PI()*(N27/1000)^2/4)</f>
-        <v/>
-      </c>
-      <c r="S29" s="455" t="n">
-        <v>16.874</v>
-      </c>
-      <c r="T29" s="455" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="U29" s="455" t="n">
-        <v>15.532</v>
-      </c>
-      <c r="V29" s="455" t="n">
-        <v>15.421</v>
-      </c>
-      <c r="W29" s="452">
-        <f>S27-U27-N27/1000</f>
-        <v/>
-      </c>
-      <c r="X29" s="452">
-        <f>T27-V27-N27/1000</f>
-        <v/>
-      </c>
-      <c r="Y29" s="452">
-        <f>P27*PI()*(N27/1000)^2/4</f>
-        <v/>
-      </c>
+      <c r="A29" s="360" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS / HYPOTHÈSES</t>
+        </is>
+      </c>
+      <c r="B29" s="351" t="n"/>
+      <c r="C29" s="352" t="n"/>
+      <c r="D29" s="353" t="n"/>
+      <c r="E29" s="354" t="n"/>
+      <c r="F29" s="331" t="n"/>
+      <c r="G29" s="354" t="n"/>
+      <c r="H29" s="354" t="n"/>
+      <c r="I29" s="354" t="n"/>
+      <c r="J29" s="331" t="n"/>
+      <c r="K29" s="331" t="n"/>
+      <c r="L29" s="355" t="n"/>
+      <c r="M29" s="356" t="n"/>
+      <c r="N29" s="325" t="n"/>
+      <c r="O29" s="357" t="n"/>
+      <c r="P29" s="353" t="n"/>
+      <c r="Q29" s="331" t="n"/>
+      <c r="R29" s="355" t="n"/>
+      <c r="S29" s="331" t="n"/>
+      <c r="T29" s="331" t="n"/>
+      <c r="U29" s="326" t="n"/>
+      <c r="V29" s="358" t="n"/>
+      <c r="W29" s="336" t="n"/>
+      <c r="X29" s="326" t="n"/>
+      <c r="Y29" s="326" t="n"/>
       <c r="Z29" s="326" t="n"/>
       <c r="AA29" s="347" t="n"/>
-      <c r="AB29" s="456">
-        <f>IF(R27&gt;L27,"OK","AUGMENTER D")</f>
-        <v/>
-      </c>
-      <c r="AC29" s="349" t="inlineStr">
-        <is>
-          <t>L11_P11_P12</t>
-        </is>
-      </c>
+      <c r="AB29" s="359" t="n"/>
     </row>
     <row r="30" ht="22.5" customHeight="1" s="206">
-      <c r="A30" s="338" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B30" s="338" t="inlineStr">
-        <is>
-          <t>@</t>
-        </is>
-      </c>
-      <c r="C30" s="338" t="inlineStr">
-        <is>
-          <t>RACC</t>
-        </is>
-      </c>
-      <c r="D30" s="448">
-        <f>D27+Q27</f>
-        <v/>
-      </c>
-      <c r="E30" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="450" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G30" s="451">
-        <f>E28*F28</f>
-        <v/>
-      </c>
-      <c r="H30" s="451">
-        <f>H27+E28</f>
-        <v/>
-      </c>
-      <c r="I30" s="451">
-        <f>I27+G28</f>
-        <v/>
-      </c>
-      <c r="J30" s="452">
-        <f>IF(H28=0,0,I28/H28)</f>
-        <v/>
-      </c>
-      <c r="K30" s="448" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D28+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D28+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D28+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D28+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D28+$S$9)^$T$9),$R$10/((D28+$S$10)^$T$10))))))</t>
-        </is>
-      </c>
-      <c r="L30" s="452">
-        <f>0.00275*H28*J28*K28</f>
-        <v/>
-      </c>
-      <c r="M30" s="449" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="N30" s="453" t="n">
-        <v>450</v>
-      </c>
-      <c r="O30" s="448">
-        <f>IF(OR(N28&lt;=0,M28&lt;=0),0,((N28/4000)^(2/3)*SQRT(M28))/$S$11)</f>
-        <v/>
-      </c>
-      <c r="P30" s="454" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="Q30" s="448">
-        <f>IF(O28=0,0,P28/(O28*60))</f>
-        <v/>
-      </c>
-      <c r="R30" s="452">
-        <f>O28*(PI()*(N28/1000)^2/4)</f>
-        <v/>
-      </c>
-      <c r="S30" s="455" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="T30" s="455" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="U30" s="455" t="n">
-        <v>15.401</v>
-      </c>
-      <c r="V30" s="455" t="n">
-        <v>15.305</v>
-      </c>
-      <c r="W30" s="452">
-        <f>S28-U28-N28/1000</f>
-        <v/>
-      </c>
-      <c r="X30" s="452">
-        <f>T28-V28-N28/1000</f>
-        <v/>
-      </c>
-      <c r="Y30" s="452">
-        <f>P28*PI()*(N28/1000)^2/4</f>
-        <v/>
-      </c>
+      <c r="A30" s="361" t="inlineStr">
+        <is>
+          <t>Jaune = saisie; Vert = calculé automatiquement (Station Saint-Hubert).</t>
+        </is>
+      </c>
+      <c r="B30" s="362" t="n"/>
+      <c r="C30" s="362" t="n"/>
+      <c r="D30" s="362" t="n"/>
+      <c r="E30" s="362" t="n"/>
+      <c r="F30" s="362" t="n"/>
+      <c r="G30" s="362" t="n"/>
+      <c r="H30" s="362" t="n"/>
+      <c r="I30" s="362" t="n"/>
+      <c r="J30" s="362" t="n"/>
+      <c r="K30" s="362" t="n"/>
+      <c r="L30" s="363" t="n"/>
+      <c r="M30" s="356" t="n"/>
+      <c r="N30" s="325" t="n"/>
+      <c r="O30" s="357" t="n"/>
+      <c r="P30" s="353" t="n"/>
+      <c r="Q30" s="331" t="n"/>
+      <c r="R30" s="355" t="n"/>
+      <c r="S30" s="331" t="n"/>
+      <c r="T30" s="331" t="n"/>
+      <c r="U30" s="326" t="n"/>
+      <c r="V30" s="358" t="n"/>
+      <c r="W30" s="336" t="n"/>
+      <c r="X30" s="326" t="n"/>
+      <c r="Y30" s="326" t="n"/>
       <c r="Z30" s="326" t="n"/>
       <c r="AA30" s="347" t="n"/>
-      <c r="AB30" s="456">
-        <f>IF(R28&gt;L28,"OK","AUGMENTER D")</f>
-        <v/>
-      </c>
-      <c r="AC30" s="349" t="inlineStr">
-        <is>
-          <t>L13_P12_RACC</t>
-        </is>
-      </c>
+      <c r="AB30" s="359" t="n"/>
     </row>
     <row r="31" ht="22.5" customHeight="1" s="206">
-      <c r="A31" s="350" t="n"/>
-      <c r="B31" s="351" t="n"/>
-      <c r="C31" s="352" t="n"/>
-      <c r="D31" s="353" t="n"/>
-      <c r="E31" s="354" t="n"/>
-      <c r="F31" s="331" t="n"/>
-      <c r="G31" s="354" t="n"/>
-      <c r="H31" s="354" t="n"/>
-      <c r="I31" s="354" t="n"/>
-      <c r="J31" s="331" t="n"/>
-      <c r="K31" s="331" t="n"/>
-      <c r="L31" s="355" t="n"/>
+      <c r="A31" s="364" t="inlineStr">
+        <is>
+          <t>Source données: Reseau_pluvial_dimensionnement_v1.xlsx (CB_plan aires, Conduites longueurs/topologie, Noeuds élévations, Inputs IDF/n/pente).</t>
+        </is>
+      </c>
+      <c r="B31" s="362" t="n"/>
+      <c r="C31" s="362" t="n"/>
+      <c r="D31" s="362" t="n"/>
+      <c r="E31" s="362" t="n"/>
+      <c r="F31" s="362" t="n"/>
+      <c r="G31" s="362" t="n"/>
+      <c r="H31" s="362" t="n"/>
+      <c r="I31" s="362" t="n"/>
+      <c r="J31" s="362" t="n"/>
+      <c r="K31" s="362" t="n"/>
+      <c r="L31" s="363" t="n"/>
       <c r="M31" s="356" t="n"/>
       <c r="N31" s="325" t="n"/>
       <c r="O31" s="357" t="n"/>
@@ -4896,7 +4491,11 @@
       <c r="AB31" s="359" t="n"/>
     </row>
     <row r="32" ht="22.5" customHeight="1" s="206">
-      <c r="A32" s="361" t="n"/>
+      <c r="A32" s="361" t="inlineStr">
+        <is>
+          <t>Qmax = 0.00275 × A(ha) × R × I   |   I = A/(tc+B)^C selon période S2 (défaut 1/10 ans).</t>
+        </is>
+      </c>
       <c r="B32" s="362" t="n"/>
       <c r="C32" s="362" t="n"/>
       <c r="D32" s="362" t="n"/>
@@ -4926,9 +4525,9 @@
       <c r="AB32" s="359" t="n"/>
     </row>
     <row r="33" ht="22.5" customHeight="1" s="206">
-      <c r="A33" s="463" t="inlineStr">
-        <is>
-          <t>INSTRUCTIONS / HYPOTHÈSES</t>
+      <c r="A33" s="364" t="inlineStr">
+        <is>
+          <t>v et Qp = Manning pleine section; n = S11 (0.013). Diamètre N est une suggestion — ajuster si AB = AUGMENTER D.</t>
         </is>
       </c>
       <c r="B33" s="362" t="n"/>
@@ -4942,7 +4541,7 @@
       <c r="J33" s="362" t="n"/>
       <c r="K33" s="362" t="n"/>
       <c r="L33" s="363" t="n"/>
-      <c r="M33" s="356" t="n"/>
+      <c r="M33" s="365" t="n"/>
       <c r="N33" s="325" t="n"/>
       <c r="O33" s="357" t="n"/>
       <c r="P33" s="353" t="n"/>
@@ -4950,349 +4549,86 @@
       <c r="R33" s="355" t="n"/>
       <c r="S33" s="331" t="n"/>
       <c r="T33" s="331" t="n"/>
-      <c r="U33" s="326" t="n"/>
+      <c r="U33" s="331" t="n"/>
       <c r="V33" s="358" t="n"/>
       <c r="W33" s="336" t="n"/>
       <c r="X33" s="326" t="n"/>
       <c r="Y33" s="326" t="n"/>
       <c r="Z33" s="326" t="n"/>
       <c r="AA33" s="347" t="n"/>
-      <c r="AB33" s="359" t="n"/>
+      <c r="AC33" s="359" t="n"/>
     </row>
     <row r="34" ht="22.5" customHeight="1" s="206">
-      <c r="A34" s="361" t="inlineStr">
-        <is>
-          <t>Jaune = saisie; Vert = calculé automatiquement (méthode simple Saint-Hubert).</t>
-        </is>
-      </c>
-      <c r="B34" s="362" t="n"/>
-      <c r="C34" s="362" t="n"/>
-      <c r="D34" s="362" t="n"/>
-      <c r="E34" s="362" t="n"/>
-      <c r="F34" s="362" t="n"/>
-      <c r="G34" s="362" t="n"/>
-      <c r="H34" s="362" t="n"/>
-      <c r="I34" s="362" t="n"/>
-      <c r="J34" s="362" t="n"/>
-      <c r="K34" s="362" t="n"/>
-      <c r="L34" s="363" t="n"/>
-      <c r="M34" s="356" t="n"/>
-      <c r="N34" s="325" t="n"/>
-      <c r="O34" s="357" t="n"/>
-      <c r="P34" s="353" t="n"/>
-      <c r="Q34" s="331" t="n"/>
-      <c r="R34" s="355" t="n"/>
-      <c r="S34" s="331" t="n"/>
-      <c r="T34" s="331" t="n"/>
-      <c r="U34" s="326" t="n"/>
-      <c r="V34" s="358" t="n"/>
-      <c r="W34" s="336" t="n"/>
-      <c r="X34" s="326" t="n"/>
-      <c r="Y34" s="326" t="n"/>
-      <c r="Z34" s="326" t="n"/>
-      <c r="AA34" s="347" t="n"/>
-      <c r="AB34" s="359" t="n"/>
+      <c r="A34" s="366" t="inlineStr">
+        <is>
+          <t>tc: temps d’entrée (Temps de concentration) puis cumul + temps de parcours Q=L/(v*60).</t>
+        </is>
+      </c>
+      <c r="B34" s="278" t="n"/>
+      <c r="C34" s="278" t="n"/>
+      <c r="D34" s="278" t="n"/>
+      <c r="E34" s="278" t="n"/>
+      <c r="F34" s="278" t="n"/>
+      <c r="G34" s="278" t="n"/>
+      <c r="H34" s="278" t="n"/>
+      <c r="I34" s="278" t="n"/>
+      <c r="J34" s="278" t="n"/>
+      <c r="K34" s="278" t="n"/>
+      <c r="L34" s="279" t="n"/>
+      <c r="M34" s="367" t="n"/>
+      <c r="N34" s="312" t="n"/>
+      <c r="O34" s="320" t="n"/>
+      <c r="P34" s="368" t="n"/>
+      <c r="Q34" s="313" t="n"/>
+      <c r="R34" s="369" t="n"/>
+      <c r="S34" s="313" t="n"/>
+      <c r="T34" s="313" t="n"/>
+      <c r="U34" s="313" t="n"/>
+      <c r="V34" s="370" t="n"/>
+      <c r="W34" s="371" t="n"/>
+      <c r="X34" s="372" t="n"/>
+      <c r="Y34" s="372" t="n"/>
+      <c r="Z34" s="372" t="n"/>
+      <c r="AA34" s="373" t="n"/>
+      <c r="AC34" s="359" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="206">
-      <c r="A35" s="364" t="inlineStr">
-        <is>
-          <t>MAJ plan: nouveau regard J01; conduite L12 P02→J01 ≈1.4 m; P03 renommé RP03; longueurs/diamètres selon plan.</t>
-        </is>
-      </c>
-      <c r="B35" s="362" t="n"/>
-      <c r="C35" s="362" t="n"/>
-      <c r="D35" s="362" t="n"/>
-      <c r="E35" s="362" t="n"/>
-      <c r="F35" s="362" t="n"/>
-      <c r="G35" s="362" t="n"/>
-      <c r="H35" s="362" t="n"/>
-      <c r="I35" s="362" t="n"/>
-      <c r="J35" s="362" t="n"/>
-      <c r="K35" s="362" t="n"/>
-      <c r="L35" s="363" t="n"/>
-      <c r="M35" s="356" t="n"/>
-      <c r="N35" s="325" t="n"/>
-      <c r="O35" s="357" t="n"/>
-      <c r="P35" s="353" t="n"/>
-      <c r="Q35" s="331" t="n"/>
-      <c r="R35" s="355" t="n"/>
-      <c r="S35" s="331" t="n"/>
-      <c r="T35" s="331" t="n"/>
-      <c r="U35" s="326" t="n"/>
-      <c r="V35" s="358" t="n"/>
-      <c r="W35" s="336" t="n"/>
-      <c r="X35" s="326" t="n"/>
-      <c r="Y35" s="326" t="n"/>
-      <c r="Z35" s="326" t="n"/>
-      <c r="AA35" s="347" t="n"/>
-      <c r="AB35" s="359" t="n"/>
+      <c r="A35" s="209" t="inlineStr">
+        <is>
+          <t>Radiers: calés depuis exutoire invert 15.305 m (Inputs), pente min 1%, chute regard 0.02 m.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="206">
-      <c r="A36" s="361" t="inlineStr">
-        <is>
-          <t>H/I: fusion correcte aux confluences. L07 et L12 = branches (H=DA locale). L08=H_L06+H_L07+DA. L02=H_L01+H_L12+DA.</t>
-        </is>
-      </c>
-      <c r="B36" s="362" t="n"/>
-      <c r="C36" s="362" t="n"/>
-      <c r="D36" s="362" t="n"/>
-      <c r="E36" s="362" t="n"/>
-      <c r="F36" s="362" t="n"/>
-      <c r="G36" s="362" t="n"/>
-      <c r="H36" s="362" t="n"/>
-      <c r="I36" s="362" t="n"/>
-      <c r="J36" s="362" t="n"/>
-      <c r="K36" s="362" t="n"/>
-      <c r="L36" s="363" t="n"/>
-      <c r="M36" s="356" t="n"/>
-      <c r="N36" s="325" t="n"/>
-      <c r="O36" s="357" t="n"/>
-      <c r="P36" s="353" t="n"/>
-      <c r="Q36" s="331" t="n"/>
-      <c r="R36" s="355" t="n"/>
-      <c r="S36" s="331" t="n"/>
-      <c r="T36" s="331" t="n"/>
-      <c r="U36" s="326" t="n"/>
-      <c r="V36" s="358" t="n"/>
-      <c r="W36" s="336" t="n"/>
-      <c r="X36" s="326" t="n"/>
-      <c r="Y36" s="326" t="n"/>
-      <c r="Z36" s="326" t="n"/>
-      <c r="AA36" s="347" t="n"/>
-      <c r="AB36" s="359" t="n"/>
+      <c r="A36" s="209" t="inlineStr">
+        <is>
+          <t>Changer la période: modifier S2 (ex. 1/25, 1/100). Les coefficients A,B,C sont dans Q5:T10.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="206">
-      <c r="A37" s="364" t="inlineStr">
-        <is>
-          <t>Qmax = 0.00275 × A(ha) × R × I   |   I = A/(tc+B)^C selon période S2.</t>
-        </is>
-      </c>
-      <c r="B37" s="362" t="n"/>
-      <c r="C37" s="362" t="n"/>
-      <c r="D37" s="362" t="n"/>
-      <c r="E37" s="362" t="n"/>
-      <c r="F37" s="362" t="n"/>
-      <c r="G37" s="362" t="n"/>
-      <c r="H37" s="362" t="n"/>
-      <c r="I37" s="362" t="n"/>
-      <c r="J37" s="362" t="n"/>
-      <c r="K37" s="362" t="n"/>
-      <c r="L37" s="363" t="n"/>
-      <c r="M37" s="365" t="n"/>
-      <c r="N37" s="325" t="n"/>
-      <c r="O37" s="357" t="n"/>
-      <c r="P37" s="353" t="n"/>
-      <c r="Q37" s="331" t="n"/>
-      <c r="R37" s="355" t="n"/>
-      <c r="S37" s="331" t="n"/>
-      <c r="T37" s="331" t="n"/>
-      <c r="U37" s="331" t="n"/>
-      <c r="V37" s="358" t="n"/>
-      <c r="W37" s="336" t="n"/>
-      <c r="X37" s="326" t="n"/>
-      <c r="Y37" s="326" t="n"/>
-      <c r="Z37" s="326" t="n"/>
-      <c r="AA37" s="347" t="n"/>
-      <c r="AC37" s="359" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="206">
-      <c r="A38" s="366" t="inlineStr">
-        <is>
-          <t>v et Qp = Manning pleine section; n = S11 (0.013). Diamètre N selon étiquettes plan.</t>
-        </is>
-      </c>
-      <c r="B38" s="278" t="n"/>
-      <c r="C38" s="278" t="n"/>
-      <c r="D38" s="278" t="n"/>
-      <c r="E38" s="278" t="n"/>
-      <c r="F38" s="278" t="n"/>
-      <c r="G38" s="278" t="n"/>
-      <c r="H38" s="278" t="n"/>
-      <c r="I38" s="278" t="n"/>
-      <c r="J38" s="278" t="n"/>
-      <c r="K38" s="278" t="n"/>
-      <c r="L38" s="279" t="n"/>
-      <c r="M38" s="367" t="n"/>
-      <c r="N38" s="312" t="n"/>
-      <c r="O38" s="320" t="n"/>
-      <c r="P38" s="368" t="n"/>
-      <c r="Q38" s="313" t="n"/>
-      <c r="R38" s="369" t="n"/>
-      <c r="S38" s="313" t="n"/>
-      <c r="T38" s="313" t="n"/>
-      <c r="U38" s="313" t="n"/>
-      <c r="V38" s="370" t="n"/>
-      <c r="W38" s="371" t="n"/>
-      <c r="X38" s="372" t="n"/>
-      <c r="Y38" s="372" t="n"/>
-      <c r="Z38" s="372" t="n"/>
-      <c r="AA38" s="373" t="n"/>
-      <c r="AC38" s="359" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="206">
-      <c r="A39" s="209" t="inlineStr">
-        <is>
-          <t>Radiers: calés depuis exutoire invert 15.305 m, pente min 1%, chute regard 0.02 m (recalculés).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="206">
-      <c r="A40" s="209" t="inlineStr">
-        <is>
-          <t>Zones L02 hist. B,C,F: B→L12 (P02); C+F→L02 (J01→RP03). Vérifier lateraux P05/P07→RP03 si conduites séparées.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="206">
-      <c r="A41" s="209" t="inlineStr">
+      <c r="A37" s="209" t="inlineStr">
         <is>
           <t>Cette feuille garde la logique simple demandée; le classeur v1 reste la référence détaillée.</t>
         </is>
       </c>
     </row>
+    <row r="38" ht="15" customHeight="1" s="206"/>
+    <row r="39" ht="15" customHeight="1" s="206"/>
+    <row r="40" ht="15" customHeight="1" s="206"/>
+    <row r="41" ht="15" customHeight="1" s="206"/>
     <row r="42" ht="15" customHeight="1" s="206"/>
     <row r="43" ht="15" customHeight="1" s="206"/>
     <row r="44" ht="15" customHeight="1" s="206"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81" ht="15" customHeight="1" s="206"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85">
-      <c r="F85" s="209" t="inlineStr">
+    <row r="81" ht="15" customHeight="1" s="206">
+      <c r="F81" s="209" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
     </row>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173" ht="15" customHeight="1" s="206"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177">
-      <c r="F177" s="209" t="inlineStr">
+    <row r="173" ht="15" customHeight="1" s="206">
+      <c r="F173" s="209" t="inlineStr">
         <is>
           <t>,0,</t>
         </is>
@@ -5339,6 +4675,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5348,7 +4685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Y119"/>
+  <dimension ref="A1:Y109"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.00390625" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19.66" customWidth="1" style="205" min="1" max="1"/>
@@ -5386,7 +4723,7 @@
       </c>
       <c r="O2" s="377" t="inlineStr">
         <is>
-          <t>Source CB_plan (v1) + plan J01/RP03. B→L12; C+F→L02.</t>
+          <t>Source CB_plan (v1). Résumé + détail zones. Tes notes L06/L07 plus bas sont conservées.</t>
         </is>
       </c>
     </row>
@@ -5467,11 +4804,7 @@
           <t>L11</t>
         </is>
       </c>
-      <c r="J5" s="385" t="inlineStr">
-        <is>
-          <t>L12</t>
-        </is>
-      </c>
+      <c r="J5" s="385" t="n"/>
       <c r="K5" s="385" t="n"/>
       <c r="L5" s="385" t="n"/>
       <c r="M5" s="386" t="n"/>
@@ -5530,7 +4863,7 @@
         <v>0.02573</v>
       </c>
       <c r="G6" s="392" t="n">
-        <v>0.034509</v>
+        <v>0.046789</v>
       </c>
       <c r="H6" s="392" t="n">
         <v>0.09030000000000001</v>
@@ -5538,9 +4871,7 @@
       <c r="I6" s="392" t="n">
         <v>0.049761</v>
       </c>
-      <c r="J6" s="457" t="n">
-        <v>0.01228</v>
-      </c>
+      <c r="J6" s="393" t="n"/>
       <c r="K6" s="393" t="n"/>
       <c r="L6" s="394" t="n"/>
       <c r="M6" s="395" t="n"/>
@@ -5607,10 +4938,7 @@
         <f>((2.187*I10*I11)/(I12)^0.5)^0.467</f>
         <v/>
       </c>
-      <c r="J7" s="458">
-        <f>((2.187*J10*J11)/(J12)^0.5)^0.467</f>
-        <v/>
-      </c>
+      <c r="J7" s="403" t="n"/>
       <c r="K7" s="403" t="n"/>
       <c r="L7" s="403" t="n"/>
       <c r="M7" s="404" t="n"/>
@@ -5665,7 +4993,7 @@
         <v>0.633</v>
       </c>
       <c r="G8" s="411" t="n">
-        <v>0.631</v>
+        <v>0.642</v>
       </c>
       <c r="H8" s="411" t="n">
         <v>0.95</v>
@@ -5673,9 +5001,7 @@
       <c r="I8" s="411" t="n">
         <v>0.335</v>
       </c>
-      <c r="J8" s="459" t="n">
-        <v>0.672</v>
-      </c>
+      <c r="J8" s="412" t="n"/>
       <c r="K8" s="412" t="n"/>
       <c r="L8" s="412" t="n"/>
       <c r="M8" s="413" t="n"/>
@@ -5765,7 +5091,7 @@
         <v>16</v>
       </c>
       <c r="G10" s="418" t="n">
-        <v>18.6</v>
+        <v>21.6</v>
       </c>
       <c r="H10" s="418" t="n">
         <v>30</v>
@@ -5773,9 +5099,7 @@
       <c r="I10" s="418" t="n">
         <v>22.3</v>
       </c>
-      <c r="J10" s="460" t="n">
-        <v>11.1</v>
-      </c>
+      <c r="J10" s="419" t="n"/>
       <c r="K10" s="419" t="n"/>
       <c r="L10" s="419" t="n"/>
       <c r="M10" s="420" t="n"/>
@@ -5834,34 +5158,32 @@
       <c r="I11" s="422" t="n">
         <v>0.02</v>
       </c>
-      <c r="J11" s="461" t="n">
-        <v>0.02</v>
-      </c>
+      <c r="J11" s="423" t="n"/>
       <c r="K11" s="423" t="n"/>
       <c r="L11" s="423" t="n"/>
       <c r="M11" s="424" t="n"/>
       <c r="N11" s="380" t="n"/>
       <c r="O11" s="396" t="inlineStr">
         <is>
-          <t>L12</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="P11" s="397" t="inlineStr">
         <is>
-          <t>B (P02→J01)</t>
+          <t>B, C, F</t>
         </is>
       </c>
       <c r="Q11" s="398" t="n">
-        <v>122.8</v>
+        <v>467.89</v>
       </c>
       <c r="R11" s="398" t="n">
-        <v>82.56999999999999</v>
+        <v>300.33</v>
       </c>
       <c r="S11" s="399" t="n">
-        <v>0.672</v>
+        <v>0.642</v>
       </c>
       <c r="T11" s="400" t="n">
-        <v>0.01228</v>
+        <v>0.0468</v>
       </c>
       <c r="U11" s="380" t="n"/>
     </row>
@@ -5872,80 +5194,78 @@
         </is>
       </c>
       <c r="B12" s="426" t="n">
-        <v>0.0308</v>
+        <v>0.03057</v>
       </c>
       <c r="C12" s="427" t="n">
-        <v>0.01</v>
+        <v>0.0041</v>
       </c>
       <c r="D12" s="427" t="n">
-        <v>0.01</v>
+        <v>0.01458</v>
       </c>
       <c r="E12" s="427" t="n">
-        <v>0.01</v>
+        <v>0.00319</v>
       </c>
       <c r="F12" s="427" t="n">
-        <v>0.01</v>
+        <v>0.00746</v>
       </c>
       <c r="G12" s="427" t="n">
-        <v>0.0104</v>
+        <v>0.01142</v>
       </c>
       <c r="H12" s="427" t="n">
-        <v>0.01</v>
+        <v>0.00628</v>
       </c>
       <c r="I12" s="427" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="J12" s="462" t="n">
-        <v>0.01</v>
-      </c>
+        <v>0.01231</v>
+      </c>
+      <c r="J12" s="428" t="n"/>
       <c r="K12" s="429" t="n"/>
       <c r="L12" s="412" t="n"/>
       <c r="M12" s="430" t="n"/>
       <c r="N12" s="431" t="n"/>
       <c r="O12" s="432" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="P12" s="400" t="inlineStr">
         <is>
-          <t>C, F (J01→RP03)</t>
+          <t>(aucune – transfert)</t>
         </is>
       </c>
       <c r="Q12" s="398" t="n">
-        <v>345.09</v>
+        <v>0</v>
       </c>
       <c r="R12" s="398" t="n">
-        <v>217.77</v>
-      </c>
-      <c r="S12" s="399" t="n">
-        <v>0.631</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="S12" s="399" t="n"/>
       <c r="T12" s="400" t="n">
-        <v>0.034509</v>
+        <v>0</v>
       </c>
       <c r="U12" s="380" t="n"/>
     </row>
     <row r="13">
       <c r="O13" s="433" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L10</t>
         </is>
       </c>
       <c r="P13" s="434" t="inlineStr">
         <is>
-          <t>(transfert RP03→P10)</t>
+          <t>N</t>
         </is>
       </c>
       <c r="Q13" s="435" t="n">
-        <v>0</v>
+        <v>903</v>
       </c>
       <c r="R13" s="435" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="436" t="n"/>
+        <v>857.85</v>
+      </c>
+      <c r="S13" s="436" t="n">
+        <v>0.95</v>
+      </c>
       <c r="T13" s="437" t="n">
-        <v>0</v>
+        <v>0.09030000000000001</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="206">
@@ -5956,25 +5276,25 @@
       </c>
       <c r="O14" s="433" t="inlineStr">
         <is>
-          <t>L10</t>
+          <t>L11</t>
         </is>
       </c>
       <c r="P14" s="434" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>O</t>
         </is>
       </c>
       <c r="Q14" s="435" t="n">
-        <v>903</v>
+        <v>497.61</v>
       </c>
       <c r="R14" s="435" t="n">
-        <v>857.85</v>
+        <v>166.52</v>
       </c>
       <c r="S14" s="436" t="n">
-        <v>0.95</v>
+        <v>0.335</v>
       </c>
       <c r="T14" s="437" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.0498</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="206">
@@ -5983,28 +5303,6 @@
           <t>Jaune = saisie (depuis Reseau_pluvial_dimensionnement_v1). Vert = calculé.</t>
         </is>
       </c>
-      <c r="O15" s="205" t="inlineStr">
-        <is>
-          <t>L11</t>
-        </is>
-      </c>
-      <c r="P15" s="205" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="Q15" s="205" t="n">
-        <v>497.61</v>
-      </c>
-      <c r="R15" s="205" t="n">
-        <v>166.52</v>
-      </c>
-      <c r="S15" s="205" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="T15" s="205" t="n">
-        <v>0.0498</v>
-      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="206">
       <c r="A16" s="205" t="inlineStr">
@@ -6014,22 +5312,8 @@
       </c>
       <c r="O16" s="438" t="inlineStr">
         <is>
-          <t>L13</t>
-        </is>
-      </c>
-      <c r="P16" s="205" t="inlineStr">
-        <is>
-          <t>(P12→RACC)</t>
-        </is>
-      </c>
-      <c r="Q16" s="205" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="205" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="205" t="n">
-        <v>0</v>
+          <t>DETAIL ZONE PAR ZONE</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="206">
@@ -6038,12 +5322,36 @@
           <t>IDF utilisée dans Calcul_reseau: période 1/10 ans (A=508.07, B=2.9, C=0.644) = Inputs du projet.</t>
         </is>
       </c>
-      <c r="O17" s="388" t="n"/>
-      <c r="P17" s="388" t="n"/>
-      <c r="Q17" s="388" t="n"/>
-      <c r="R17" s="388" t="n"/>
-      <c r="S17" s="388" t="n"/>
-      <c r="T17" s="388" t="n"/>
+      <c r="O17" s="388" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="P17" s="388" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="Q17" s="388" t="inlineStr">
+        <is>
+          <t>Roof m²</t>
+        </is>
+      </c>
+      <c r="R17" s="388" t="inlineStr">
+        <is>
+          <t>Pave m²</t>
+        </is>
+      </c>
+      <c r="S17" s="388" t="inlineStr">
+        <is>
+          <t>Grass m²</t>
+        </is>
+      </c>
+      <c r="T17" s="388" t="inlineStr">
+        <is>
+          <t>Other m²</t>
+        </is>
+      </c>
       <c r="U17" s="388" t="inlineStr">
         <is>
           <t>A m²</t>
@@ -7237,21 +6545,21 @@
       </c>
       <c r="B57" s="442" t="inlineStr">
         <is>
-          <t>15.6 m</t>
+          <t>15.7 m</t>
         </is>
       </c>
     </row>
     <row r="58" ht="31.9" customHeight="1" s="206">
       <c r="A58" s="442" t="inlineStr">
         <is>
-          <t>s = (17.62 - 17.14) / 15.6</t>
+          <t>s = (17.62 - 17.14) / 15.7</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="206">
       <c r="A59" s="442" t="inlineStr">
         <is>
-          <t xml:space="preserve"> s = 0.48 / 15.6</t>
+          <t xml:space="preserve"> s = 0.48 / 15.7</t>
         </is>
       </c>
     </row>
@@ -7262,7 +6570,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="376" t="inlineStr">
         <is>
@@ -7270,7 +6577,6 @@
         </is>
       </c>
     </row>
-    <row r="63"/>
     <row r="64">
       <c r="A64" s="447" t="inlineStr">
         <is>
@@ -7279,7 +6585,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="205" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>Zones G:</t>
         </is>
@@ -7376,13 +6682,12 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="205" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>C = 101.1300 / 147.90 = 0.6838</t>
         </is>
       </c>
     </row>
-    <row r="70"/>
     <row r="71">
       <c r="A71" s="447" t="inlineStr">
         <is>
@@ -7391,7 +6696,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="205" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>Zones D:</t>
         </is>
@@ -7488,22 +6793,21 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="205" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>C = 51.7050 / 94.50 = 0.5471</t>
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="447" t="inlineStr">
         <is>
-          <t>L01_P01_J01 → A = 257.30 m², C ≈ 0.633</t>
+          <t>L01_P01_P02 → A = 257.30 m², C ≈ 0.633</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="205" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>Zones A, E:</t>
         </is>
@@ -7628,24 +6932,23 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="205" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>C = 162.8000 / 257.30 = 0.6327</t>
         </is>
       </c>
     </row>
-    <row r="85"/>
     <row r="86">
       <c r="A86" s="447" t="inlineStr">
         <is>
-          <t>L02_J01_RRP03 → A = 467.89 m², C ≈ 0.642</t>
+          <t>L02_P02_P03 → A = 467.89 m², C ≈ 0.642</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="205" t="inlineStr">
-        <is>
-          <t>Zones historiques B,C,F — ventilées: B→L12 (P02→J01); C+F→L02 (J01→RP03)</t>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Zones B, C, F:</t>
         </is>
       </c>
     </row>
@@ -7796,21 +7099,19 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="205" t="inlineStr">
+      <c r="A93" t="inlineStr">
         <is>
           <t>C = 300.3310 / 467.89 = 0.6419</t>
         </is>
       </c>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="447" t="inlineStr">
         <is>
-          <t>L03_RRP03_P10 → A = 0 m² (aucune zone CB — conduite de transfert)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96"/>
+          <t>L03_P03_P10 → A = 0 m² (aucune zone CB — conduite de transfert)</t>
+        </is>
+      </c>
+    </row>
     <row r="97">
       <c r="A97" s="447" t="inlineStr">
         <is>
@@ -7819,7 +7120,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="205" t="inlineStr">
+      <c r="A98" t="inlineStr">
         <is>
           <t>Zones N:</t>
         </is>
@@ -7916,13 +7217,12 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="205" t="inlineStr">
+      <c r="A102" t="inlineStr">
         <is>
           <t>C = 857.8500 / 903.00 = 0.9500</t>
         </is>
       </c>
     </row>
-    <row r="103"/>
     <row r="104">
       <c r="A104" s="447" t="inlineStr">
         <is>
@@ -7931,7 +7231,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="205" t="inlineStr">
+      <c r="A105" t="inlineStr">
         <is>
           <t>Zones O:</t>
         </is>
@@ -8028,52 +7328,12 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="205" t="inlineStr">
+      <c r="A109" t="inlineStr">
         <is>
           <t>C = 166.5225 / 497.61 = 0.3346</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="205" t="inlineStr">
-        <is>
-          <t>L12_P02_J01 (nouvelle) → A = 122.80 m² (zone B), C ≈ 0.672; L ≈ 1.4 m</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="205" t="inlineStr">
-        <is>
-          <t>Fusion J01: H(L02)=H(L01)+H(L12)+DA(L02). Ne pas cumuler L12 dans L01.</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="205" t="inlineStr">
-        <is>
-          <t>Longueurs plan: L06=15.6; L07=10.9; L08=15.2; L09=13.9; L01=14.2; L12=1.4; L02=10.6; L03=8.9; L10=14.5; L11=11.1; L13=9.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="205" t="inlineStr">
-        <is>
-          <t>Diamètres plan: L06 Ø200; L07/L08/L09 Ø250; L01/L12/L02 Ø300; L03/L10 Ø375; L11/L13 Ø450</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="205" t="inlineStr">
-        <is>
-          <t>P03 renommé RP03. Lateraux plan P05→RP03 (10.5 m) et P07→RP03 (25.4 m): non modélisés comme branches séparées — à confirmer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
   </sheetData>
   <mergeCells count="24">
     <mergeCell ref="A30:H30"/>

</xml_diff>